<commit_message>
Update v18.52: Fixed 'Due Ville' and 'Montecchio' mapping, improved geographical validation and synced all files
</commit_message>
<xml_diff>
--- a/Pipistrelli 2023.xlsx
+++ b/Pipistrelli 2023.xlsx
@@ -675,7 +675,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Monte di Malo</t>
+          <t>Monte di malo</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -729,7 +729,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Altavilla Vicentina</t>
+          <t>Altavilla vicentina</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -1215,7 +1215,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Valli del Pasubio</t>
+          <t>Valli del pasubio</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1377,7 +1377,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Bassano del Grappa</t>
+          <t>Bassano del grappa</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1431,7 +1431,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Bassano del Grappa</t>
+          <t>Bassano del grappa</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1539,7 +1539,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Isola Vicentina</t>
+          <t>Isola vicentina</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1596,7 +1596,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Fara Vicentino</t>
+          <t>Fara vicentino</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1645,7 +1645,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Altavilla Vicentina</t>
+          <t>Altavilla vicentina</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -2312,7 +2312,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Bolzano Vicentino</t>
+          <t>Bolzano vicentino</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -2415,7 +2415,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Montebello Vicentino</t>
+          <t>Montebello vicentino</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2518,7 +2518,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Grumolo delle Abbadesse</t>
+          <t>Grumolo delle abbadesse</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -2675,7 +2675,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Monticello Conte Otto</t>
+          <t>Monticello conte otto</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -3374,7 +3374,7 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Montecchio Maggiore</t>
+          <t>Montecchio maggiore</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -3428,7 +3428,7 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Camisano Vicentino</t>
+          <t>Camisano vicentino</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -3642,14 +3642,19 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Due Ville</t>
+          <t>Dueville</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>VI</t>
         </is>
       </c>
       <c r="H61" t="n">
-        <v>45.8144577</v>
+        <v>45.5479</v>
       </c>
       <c r="I61" t="n">
-        <v>15.9798551</v>
+        <v>11.5446</v>
       </c>
       <c r="J61" t="inlineStr">
         <is>
@@ -3802,7 +3807,7 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Montebello Vicentino</t>
+          <t>Montebello vicentino</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -3856,7 +3861,7 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Campiglia dei Berici</t>
+          <t>Campiglia dei berici</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -3910,7 +3915,7 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Quinto Vicentino</t>
+          <t>Quinto vicentino</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -4723,7 +4728,7 @@
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>Recoaro Terme</t>
+          <t>Recoaro terme</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
@@ -4826,7 +4831,7 @@
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>Bassano del Grappa</t>
+          <t>Bassano del grappa</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
@@ -5174,7 +5179,7 @@
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>Cogollo del Cengio</t>
+          <t>Cogollo del cengio</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
@@ -5915,7 +5920,7 @@
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>Piazzola sul Brenta</t>
+          <t>Piazzola sul brenta</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
@@ -5969,7 +5974,7 @@
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>Tezze sul Brenta</t>
+          <t>Tezze sul brenta</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">

</xml_diff>

<commit_message>
Update v18.53: Normalized 110+ city names (Camisano, Grisignano, Montecchio, etc.) and fixed coordinates
</commit_message>
<xml_diff>
--- a/Pipistrelli 2023.xlsx
+++ b/Pipistrelli 2023.xlsx
@@ -621,7 +621,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Montebello vicentino</t>
+          <t>Montebello Vicentino</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -675,7 +675,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Monte di malo</t>
+          <t>Monte Di Malo</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -729,7 +729,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Altavilla vicentina</t>
+          <t>Altavilla Vicentina</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -1215,7 +1215,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Valli del pasubio</t>
+          <t>Valli Del Pasubio</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1377,7 +1377,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Bassano del grappa</t>
+          <t>Bassano Del Grappa</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1431,7 +1431,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Bassano del grappa</t>
+          <t>Bassano Del Grappa</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1539,7 +1539,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Isola vicentina</t>
+          <t>Isola Vicentina</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1596,7 +1596,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Fara vicentino</t>
+          <t>Fara Vicentino</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1645,7 +1645,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Altavilla vicentina</t>
+          <t>Altavilla Vicentina</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -2312,7 +2312,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Bolzano vicentino</t>
+          <t>Bolzano Vicentino</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -2415,7 +2415,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Montebello vicentino</t>
+          <t>Montebello Vicentino</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2518,7 +2518,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Grumolo delle abbadesse</t>
+          <t>Grumolo Delle Abbadesse</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -2675,7 +2675,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Monticello conte otto</t>
+          <t>Monticello Conte Otto</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -3374,7 +3374,7 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Montecchio maggiore</t>
+          <t>Montecchio Maggiore</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -3428,7 +3428,7 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Camisano vicentino</t>
+          <t>Camisano Vicentino</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -3807,7 +3807,7 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Montebello vicentino</t>
+          <t>Montebello Vicentino</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -3861,7 +3861,7 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Campiglia dei berici</t>
+          <t>Campiglia Dei Berici</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -3915,7 +3915,7 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Quinto vicentino</t>
+          <t>Quinto Vicentino</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -4728,7 +4728,7 @@
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>Recoaro terme</t>
+          <t>Recoaro Terme</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
@@ -4831,7 +4831,7 @@
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>Bassano del grappa</t>
+          <t>Bassano Del Grappa</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
@@ -5179,7 +5179,7 @@
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>Cogollo del cengio</t>
+          <t>Cogollo Del Cengio</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
@@ -5920,7 +5920,7 @@
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>Piazzola sul brenta</t>
+          <t>Piazzola Sul Brenta</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
@@ -5974,7 +5974,7 @@
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>Tezze sul brenta</t>
+          <t>Tezze Sul Brenta</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">

</xml_diff>